<commit_message>
work with main file(start create vk bot)
</commit_message>
<xml_diff>
--- a/services/cards.xlsx
+++ b/services/cards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python Project\services\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28AC793-1278-4644-AC2D-7F8C35470603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49AFD0E0-6BBA-40EF-A9DB-F4032EC2B633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="15" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cards" sheetId="1" r:id="rId1"/>
@@ -64,9 +64,6 @@
     <t>обычная капибара</t>
   </si>
   <si>
-    <t>Редкость(1 - 3)</t>
-  </si>
-  <si>
     <t>ТИП</t>
   </si>
   <si>
@@ -155,18 +152,29 @@
   </si>
   <si>
     <t xml:space="preserve"> @___ @    U^ｪ^U</t>
+  </si>
+  <si>
+    <t>Редкость</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -231,26 +239,29 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -754,32 +765,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -816,7 +827,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>3</v>
@@ -932,7 +943,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>13</v>
@@ -953,7 +964,7 @@
         <v>70</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -964,7 +975,7 @@
         <v>8</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8">
         <v>2</v>
@@ -982,7 +993,7 @@
         <v>200</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="16.5">
@@ -993,7 +1004,7 @@
         <v>5</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -1022,7 +1033,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1048,10 +1059,10 @@
         <v>2</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1069,7 +1080,7 @@
         <v>300</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1077,10 +1088,10 @@
         <v>2</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1098,7 +1109,7 @@
         <v>250</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1109,7 +1120,7 @@
         <v>8</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D13">
         <v>2</v>
@@ -1135,10 +1146,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="D14">
         <v>35</v>
@@ -1164,10 +1175,10 @@
         <v>3</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1185,7 +1196,7 @@
         <v>800</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1193,10 +1204,10 @@
         <v>3</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1222,10 +1233,10 @@
         <v>3</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D17">
         <v>2</v>
@@ -1243,7 +1254,7 @@
         <v>700</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1251,10 +1262,10 @@
         <v>3</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1272,7 +1283,7 @@
         <v>750</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
start work on shop(all work mb)
</commit_message>
<xml_diff>
--- a/services/cards.xlsx
+++ b/services/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python Project\services\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{478EA938-87A2-462F-9831-330225D606DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E025E5B2-2C72-44AD-AF51-3B9EB637EE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4695" yWindow="1800" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -133,51 +133,43 @@
     <t>_|¦|_   / * &gt;</t>
   </si>
   <si>
-    <t>_/□\\_   ʕ•ᴥ•ʔ</t>
-  </si>
-  <si>
-    <t>/\/\   ( •·•)</t>
-  </si>
-  <si>
-    <t>/) /)   ( • ,•)</t>
-  </si>
-  <si>
-    <t>△   /   * )</t>
-  </si>
-  <si>
-    <t>()____()   (^(oo)^)</t>
-  </si>
-  <si>
-    <t>_|¯|_     (°)#))&lt;&lt;</t>
-  </si>
-  <si>
-    <t>_/‾\_   U'ᴥ'U</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> @___ @   U^ｪ^U</t>
-  </si>
-  <si>
-    <t>_|¦|_  / * &gt;</t>
+    <t>_/□\\_    ʕ•ᴥ•ʔ</t>
+  </si>
+  <si>
+    <t>/\/\    ( •·•)</t>
+  </si>
+  <si>
+    <t>/) /)    ( • ,•)</t>
+  </si>
+  <si>
+    <t>()____()     (^(oo)^)</t>
+  </si>
+  <si>
+    <t>△    /   * )</t>
+  </si>
+  <si>
+    <t>_|¯|_      (°)#))&lt;&lt;</t>
+  </si>
+  <si>
+    <t>_|¦|_    / * &gt;</t>
+  </si>
+  <si>
+    <t>_/‾\_    U'ᴥ'U</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> @___ @    U^ｪ^U</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -250,29 +242,26 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -920,7 +909,7 @@
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:9" s="1" customFormat="1" ht="14.25" customHeight="1">
@@ -948,8 +937,8 @@
       <c r="H6">
         <v>0</v>
       </c>
-      <c r="I6" s="9" t="s">
-        <v>45</v>
+      <c r="I6" s="8" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -978,7 +967,7 @@
         <v>70</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1007,7 +996,7 @@
         <v>200</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="16.5">
@@ -1094,7 +1083,7 @@
         <v>300</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1152,7 +1141,7 @@
         <v>450</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1210,7 +1199,7 @@
         <v>800</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1297,7 +1286,7 @@
         <v>750</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correct reg with adding 5 sparrow after it
</commit_message>
<xml_diff>
--- a/services/cards.xlsx
+++ b/services/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python Project\services\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A79AD13-2F3A-42AD-8F86-D1B13894D523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA75CE4-9BAE-41F2-A28B-D54C0F4E5928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4695" yWindow="1800" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="47">
   <si>
     <t>security</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t xml:space="preserve">  @___ @    U^ｪ^U</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> /\/\   ( •·•)</t>
   </si>
 </sst>
 </file>
@@ -851,7 +854,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:9">

</xml_diff>

<commit_message>
start work on shop(check excel tab and names in shop rep)
</commit_message>
<xml_diff>
--- a/services/cards.xlsx
+++ b/services/cards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python Project\services\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA75CE4-9BAE-41F2-A28B-D54C0F4E5928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43F271F-C36C-4C25-9CC1-4E537F85EBB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4695" yWindow="1800" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8865" yWindow="5940" windowWidth="28800" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cards" sheetId="1" r:id="rId1"/>
@@ -822,7 +822,7 @@
         <v>4</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="I2" t="s">
         <v>35</v>
@@ -851,7 +851,7 @@
         <v>3</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I3" t="s">
         <v>46</v>
@@ -880,7 +880,7 @@
         <v>3</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I4" t="s">
         <v>37</v>
@@ -909,7 +909,7 @@
         <v>2</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I5" t="s">
         <v>38</v>
@@ -938,7 +938,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
work on vkapi(dont show main menu)
</commit_message>
<xml_diff>
--- a/services/cards.xlsx
+++ b/services/cards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python Project\services\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4974864A-28CA-437F-B066-963E0A5BF999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E628C6-B3DE-42B8-98F5-62EF521FD8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3855" yWindow="5250" windowWidth="30120" windowHeight="14070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cards" sheetId="1" r:id="rId1"/>

</xml_diff>